<commit_message>
Sổ tổ trưởng: sửa file xuất bị Excel báo lỗi (vùng in $NaN trong mẫu)
- Mẫu so_to_truong.xlsx mang 24 tên vùng in/tiêu đề in hỏng -> bỏ khỏi mẫu
- Dựng sổ xong đặt lại vùng in theo nội dung thật (T*: A:V, Mủ dây/đất: A:N, TỔNG: A:P)
- Chốt chặn chung khi xuất theo mẫu: vùng in / tiêu đề in không hợp lệ thì bỏ

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mau/so_to_truong.xlsx
+++ b/mau/so_to_truong.xlsx
@@ -30,32 +30,6 @@
     <sheet sheetId="9" name="TỔNG" state="visible" r:id="rId24"/>
     <sheet sheetId="4" name="Sheet5" state="visible" r:id="rId25"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'T1'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'T1'!$208:$213</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'T2'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'T2'!$196:$201</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'T3'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="11">'T3'!$194:$199</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="12">'T4'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="12">'T4'!$203:$208</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="13">'T5'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="13">'T5'!$218:$223</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="14">'T6'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="14">'T6'!$211:$216</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="15">'T7'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="15">'T7'!$199:$204</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="16">'T8'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="16">'T8'!$198:$203</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="17">'T9'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="17">'T9'!$198:$203</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="18">'Mủ đất'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="18">'Mủ đất'!$500:$505</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="19">'Mủ dây'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="19">'Mủ dây'!$501:$506</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="20">'TỔNG'!$NaN:$NaN</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="20">'TỔNG'!$533:$538</definedName>
-  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>

</xml_diff>